<commit_message>
Add shared final status Excel runtime sync
</commit_message>
<xml_diff>
--- a/docs/balance/final status.xlsx
+++ b/docs/balance/final status.xlsx
@@ -2,26 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_版本与口径" sheetId="1" r:id="Rc77e7b895931489e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_棋子基础" sheetId="2" r:id="R3813da0535534520"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_棋子技能" sheetId="3" r:id="Rbe5498b7547042b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_宠物与商城" sheetId="4" r:id="R5478ddca75cb4516"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_羁绊" sheetId="5" r:id="R693beae0369c4825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_野怪" sheetId="6" r:id="R0a2aa50d82904c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Boss" sheetId="7" r:id="R28ee6b2848364c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_佣兵" sheetId="8" r:id="R0083492c362e4e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_法阵友军" sheetId="9" r:id="R898e5e33d38a4a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_宝藏与套装" sheetId="10" r:id="R5635d0c7a93b4d68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_宝藏联动" sheetId="11" r:id="R404fd7bf1399459f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_金币规则" sheetId="12" r:id="R6631ee625a644dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_萝卜规则" sheetId="13" r:id="Rd7f7ab2fe03c4524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_回合与商店" sheetId="14" r:id="R790ad9756a3042d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_界面映射" sheetId="15" r:id="Rb74e9d730c594b0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_冲突与验证" sheetId="16" r:id="Rc2d99fefb9454534"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90_运行配置" sheetId="17" r:id="R85e91f8bcef34650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="91_来源清单" sheetId="18" r:id="Rdbcb52a0e48c418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="92_代码参数" sheetId="19" r:id="R80f2eefdfbbf4dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="93_商城目录" sheetId="20" r:id="Rf8c697e7726b4a2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_版本与口径" sheetId="1" r:id="Rbc9f94533e1f4de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_棋子基础" sheetId="2" r:id="R8c12b76d00474b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_棋子技能" sheetId="3" r:id="Rdec20b56cd0b49f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_宠物与商城" sheetId="4" r:id="Rf5fdc2bc53c84dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_羁绊" sheetId="5" r:id="Rc1e798b18c3b4964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_野怪" sheetId="6" r:id="R40effd7421f94fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Boss" sheetId="7" r:id="R859b5958df554f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_佣兵" sheetId="8" r:id="Rc421c76db5004995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_法阵友军" sheetId="9" r:id="R468702f519b34c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_宝藏与套装" sheetId="10" r:id="Rb0bd05e7ce684546"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_宝藏联动" sheetId="11" r:id="Re82476d1f1bd4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_金币规则" sheetId="12" r:id="Rc0db4d14e2014fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_萝卜规则" sheetId="13" r:id="R95cb57068bf14711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_回合与商店" sheetId="14" r:id="R6e76ca46b3e34806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_界面映射" sheetId="15" r:id="Rc5550d3bb1664009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_冲突与验证" sheetId="16" r:id="R9855aaa9e6894675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90_运行配置" sheetId="17" r:id="R136561bd0a1c4796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="91_来源清单" sheetId="18" r:id="Ra374f73a99054af8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="92_代码参数" sheetId="19" r:id="R92c8508dc14d4631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="93_商城目录" sheetId="20" r:id="R7cc36b6846f446d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4691,7 +4691,7 @@
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>高级字段：完整收录当前 Godot/商城运行 JSON。路径以 $ 为根，值按 JSON 语法编辑；普通数值优先在前面的业务页修改。导出工具会检查并生成运行文件。</x:v>
+        <x:v>历史配置快照，仅供查阅，不再参与运行前同步。基础数值以 01/03/05/06/08 业务页为准；其余复杂字段以项目中的 JSON / GDScript 为准。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -52028,7 +52028,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>40 名棋子。1–4★ HP / 攻击 / 防御为新表中的本机战斗运行值；战斗内其他加成仍按对应规则动态结算。</x:v>
+        <x:v>编辑 1★ HP / 攻击 / 防御（G、K、O 列）；2–4★由公式按游戏星级倍率计算。运行前执行 tools/run_with_final.py，同步 JSON 和游戏显示。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -52171,36 +52171,45 @@
         <x:v>580</x:v>
       </x:c>
       <x:c r="H4" s="11" t="n">
+        <x:f>ROUND(G4*1.5,0)</x:f>
         <x:v>870</x:v>
       </x:c>
       <x:c r="I4" s="11" t="n">
+        <x:f>ROUND(G4*3,0)</x:f>
         <x:v>1740</x:v>
       </x:c>
       <x:c r="J4" s="11" t="n">
+        <x:f>ROUND(G4*(3*1.15),0)</x:f>
         <x:v>2001</x:v>
       </x:c>
       <x:c r="K4" s="11" t="n">
         <x:v>37</x:v>
       </x:c>
       <x:c r="L4" s="11" t="n">
+        <x:f>ROUND(K4*1.5,0)</x:f>
         <x:v>56</x:v>
       </x:c>
       <x:c r="M4" s="11" t="n">
+        <x:f>ROUND(K4*3,0)</x:f>
         <x:v>111</x:v>
       </x:c>
       <x:c r="N4" s="11" t="n">
+        <x:f>ROUND(K4*(3*1.15),0)</x:f>
         <x:v>128</x:v>
       </x:c>
       <x:c r="O4" s="11" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P4" s="11" t="n">
+        <x:f>ROUND(O4*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q4" s="11" t="n">
+        <x:f>ROUND(O4*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R4" s="11" t="n">
+        <x:f>ROUND(O4*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S4" s="11" t="n">
@@ -52258,36 +52267,45 @@
         <x:v>520</x:v>
       </x:c>
       <x:c r="H5" s="15" t="n">
+        <x:f>ROUND(G5*1.5,0)</x:f>
         <x:v>780</x:v>
       </x:c>
       <x:c r="I5" s="15" t="n">
+        <x:f>ROUND(G5*3,0)</x:f>
         <x:v>1560</x:v>
       </x:c>
       <x:c r="J5" s="15" t="n">
+        <x:f>ROUND(G5*(3*1.15),0)</x:f>
         <x:v>1794</x:v>
       </x:c>
       <x:c r="K5" s="15" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="L5" s="15" t="n">
+        <x:f>ROUND(K5*1.5,0)</x:f>
         <x:v>72</x:v>
       </x:c>
       <x:c r="M5" s="15" t="n">
+        <x:f>ROUND(K5*3,0)</x:f>
         <x:v>144</x:v>
       </x:c>
       <x:c r="N5" s="15" t="n">
+        <x:f>ROUND(K5*(3*1.15),0)</x:f>
         <x:v>166</x:v>
       </x:c>
       <x:c r="O5" s="15" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="P5" s="15" t="n">
+        <x:f>ROUND(O5*1.5,0)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q5" s="15" t="n">
+        <x:f>ROUND(O5*3,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="R5" s="15" t="n">
+        <x:f>ROUND(O5*(3*1.15),0)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="S5" s="15" t="n">
@@ -52345,36 +52363,45 @@
         <x:v>840</x:v>
       </x:c>
       <x:c r="H6" s="11" t="n">
+        <x:f>ROUND(G6*1.5,0)</x:f>
         <x:v>1260</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
+        <x:f>ROUND(G6*3,0)</x:f>
         <x:v>2520</x:v>
       </x:c>
       <x:c r="J6" s="11" t="n">
+        <x:f>ROUND(G6*(3*1.15),0)</x:f>
         <x:v>2898</x:v>
       </x:c>
       <x:c r="K6" s="11" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="L6" s="11" t="n">
+        <x:f>ROUND(K6*1.5,0)</x:f>
         <x:v>83</x:v>
       </x:c>
       <x:c r="M6" s="11" t="n">
+        <x:f>ROUND(K6*3,0)</x:f>
         <x:v>165</x:v>
       </x:c>
       <x:c r="N6" s="11" t="n">
+        <x:f>ROUND(K6*(3*1.15),0)</x:f>
         <x:v>190</x:v>
       </x:c>
       <x:c r="O6" s="11" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="P6" s="11" t="n">
+        <x:f>ROUND(O6*1.5,0)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="Q6" s="11" t="n">
+        <x:f>ROUND(O6*3,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="R6" s="11" t="n">
+        <x:f>ROUND(O6*(3*1.15),0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="S6" s="11" t="n">
@@ -52432,36 +52459,45 @@
         <x:v>920</x:v>
       </x:c>
       <x:c r="H7" s="15" t="n">
+        <x:f>ROUND(G7*1.5,0)</x:f>
         <x:v>1380</x:v>
       </x:c>
       <x:c r="I7" s="15" t="n">
+        <x:f>ROUND(G7*3,0)</x:f>
         <x:v>2760</x:v>
       </x:c>
       <x:c r="J7" s="15" t="n">
+        <x:f>ROUND(G7*(3*1.15),0)</x:f>
         <x:v>3174</x:v>
       </x:c>
       <x:c r="K7" s="15" t="n">
         <x:v>68</x:v>
       </x:c>
       <x:c r="L7" s="15" t="n">
+        <x:f>ROUND(K7*1.5,0)</x:f>
         <x:v>102</x:v>
       </x:c>
       <x:c r="M7" s="15" t="n">
+        <x:f>ROUND(K7*3,0)</x:f>
         <x:v>204</x:v>
       </x:c>
       <x:c r="N7" s="15" t="n">
+        <x:f>ROUND(K7*(3*1.15),0)</x:f>
         <x:v>235</x:v>
       </x:c>
       <x:c r="O7" s="15" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="P7" s="15" t="n">
+        <x:f>ROUND(O7*1.5,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="Q7" s="15" t="n">
+        <x:f>ROUND(O7*3,0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="R7" s="15" t="n">
+        <x:f>ROUND(O7*(3*1.15),0)</x:f>
         <x:v>28</x:v>
       </x:c>
       <x:c r="S7" s="15" t="n">
@@ -52519,36 +52555,45 @@
         <x:v>780</x:v>
       </x:c>
       <x:c r="H8" s="11" t="n">
+        <x:f>ROUND(G8*1.5,0)</x:f>
         <x:v>1170</x:v>
       </x:c>
       <x:c r="I8" s="11" t="n">
+        <x:f>ROUND(G8*3,0)</x:f>
         <x:v>2340</x:v>
       </x:c>
       <x:c r="J8" s="11" t="n">
+        <x:f>ROUND(G8*(3*1.15),0)</x:f>
         <x:v>2691</x:v>
       </x:c>
       <x:c r="K8" s="11" t="n">
         <x:v>88</x:v>
       </x:c>
       <x:c r="L8" s="11" t="n">
+        <x:f>ROUND(K8*1.5,0)</x:f>
         <x:v>132</x:v>
       </x:c>
       <x:c r="M8" s="11" t="n">
+        <x:f>ROUND(K8*3,0)</x:f>
         <x:v>264</x:v>
       </x:c>
       <x:c r="N8" s="11" t="n">
+        <x:f>ROUND(K8*(3*1.15),0)</x:f>
         <x:v>304</x:v>
       </x:c>
       <x:c r="O8" s="11" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="P8" s="11" t="n">
+        <x:f>ROUND(O8*1.5,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="Q8" s="11" t="n">
+        <x:f>ROUND(O8*3,0)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="R8" s="11" t="n">
+        <x:f>ROUND(O8*(3*1.15),0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="S8" s="11" t="n">
@@ -52606,36 +52651,45 @@
         <x:v>860</x:v>
       </x:c>
       <x:c r="H9" s="15" t="n">
+        <x:f>ROUND(G9*1.5,0)</x:f>
         <x:v>1290</x:v>
       </x:c>
       <x:c r="I9" s="15" t="n">
+        <x:f>ROUND(G9*3,0)</x:f>
         <x:v>2580</x:v>
       </x:c>
       <x:c r="J9" s="15" t="n">
+        <x:f>ROUND(G9*(3*1.15),0)</x:f>
         <x:v>2967</x:v>
       </x:c>
       <x:c r="K9" s="15" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="L9" s="15" t="n">
+        <x:f>ROUND(K9*1.5,0)</x:f>
         <x:v>96</x:v>
       </x:c>
       <x:c r="M9" s="15" t="n">
+        <x:f>ROUND(K9*3,0)</x:f>
         <x:v>192</x:v>
       </x:c>
       <x:c r="N9" s="15" t="n">
+        <x:f>ROUND(K9*(3*1.15),0)</x:f>
         <x:v>221</x:v>
       </x:c>
       <x:c r="O9" s="15" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="P9" s="15" t="n">
+        <x:f>ROUND(O9*1.5,0)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="Q9" s="15" t="n">
+        <x:f>ROUND(O9*3,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="R9" s="15" t="n">
+        <x:f>ROUND(O9*(3*1.15),0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="S9" s="15" t="n">
@@ -52693,36 +52747,45 @@
         <x:v>1640</x:v>
       </x:c>
       <x:c r="H10" s="11" t="n">
+        <x:f>ROUND(G10*1.5,0)</x:f>
         <x:v>2460</x:v>
       </x:c>
       <x:c r="I10" s="11" t="n">
+        <x:f>ROUND(G10*3,0)</x:f>
         <x:v>4920</x:v>
       </x:c>
       <x:c r="J10" s="11" t="n">
+        <x:f>ROUND(G10*(3*1.15),0)</x:f>
         <x:v>5658</x:v>
       </x:c>
       <x:c r="K10" s="11" t="n">
         <x:v>97</x:v>
       </x:c>
       <x:c r="L10" s="11" t="n">
+        <x:f>ROUND(K10*1.5,0)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="M10" s="11" t="n">
+        <x:f>ROUND(K10*3,0)</x:f>
         <x:v>291</x:v>
       </x:c>
       <x:c r="N10" s="11" t="n">
+        <x:f>ROUND(K10*(3*1.15),0)</x:f>
         <x:v>335</x:v>
       </x:c>
       <x:c r="O10" s="11" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="P10" s="11" t="n">
+        <x:f>ROUND(O10*1.5,0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="Q10" s="11" t="n">
+        <x:f>ROUND(O10*3,0)</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="R10" s="11" t="n">
+        <x:f>ROUND(O10*(3*1.15),0)</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="S10" s="11" t="n">
@@ -52782,36 +52845,45 @@
         <x:v>1800</x:v>
       </x:c>
       <x:c r="H11" s="15" t="n">
+        <x:f>ROUND(G11*1.5,0)</x:f>
         <x:v>2700</x:v>
       </x:c>
       <x:c r="I11" s="15" t="n">
+        <x:f>ROUND(G11*3,0)</x:f>
         <x:v>5400</x:v>
       </x:c>
       <x:c r="J11" s="15" t="n">
+        <x:f>ROUND(G11*(3*1.15),0)</x:f>
         <x:v>6210</x:v>
       </x:c>
       <x:c r="K11" s="15" t="n">
         <x:v>110</x:v>
       </x:c>
       <x:c r="L11" s="15" t="n">
+        <x:f>ROUND(K11*1.5,0)</x:f>
         <x:v>165</x:v>
       </x:c>
       <x:c r="M11" s="15" t="n">
+        <x:f>ROUND(K11*3,0)</x:f>
         <x:v>330</x:v>
       </x:c>
       <x:c r="N11" s="15" t="n">
+        <x:f>ROUND(K11*(3*1.15),0)</x:f>
         <x:v>379</x:v>
       </x:c>
       <x:c r="O11" s="15" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="P11" s="15" t="n">
+        <x:f>ROUND(O11*1.5,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="Q11" s="15" t="n">
+        <x:f>ROUND(O11*3,0)</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="R11" s="15" t="n">
+        <x:f>ROUND(O11*(3*1.15),0)</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="S11" s="15" t="n">
@@ -52871,36 +52943,45 @@
         <x:v>640</x:v>
       </x:c>
       <x:c r="H12" s="11" t="n">
+        <x:f>ROUND(G12*1.5,0)</x:f>
         <x:v>960</x:v>
       </x:c>
       <x:c r="I12" s="11" t="n">
+        <x:f>ROUND(G12*3,0)</x:f>
         <x:v>1920</x:v>
       </x:c>
       <x:c r="J12" s="11" t="n">
+        <x:f>ROUND(G12*(3*1.15),0)</x:f>
         <x:v>2208</x:v>
       </x:c>
       <x:c r="K12" s="11" t="n">
         <x:v>31</x:v>
       </x:c>
       <x:c r="L12" s="11" t="n">
+        <x:f>ROUND(K12*1.5,0)</x:f>
         <x:v>47</x:v>
       </x:c>
       <x:c r="M12" s="11" t="n">
+        <x:f>ROUND(K12*3,0)</x:f>
         <x:v>93</x:v>
       </x:c>
       <x:c r="N12" s="11" t="n">
+        <x:f>ROUND(K12*(3*1.15),0)</x:f>
         <x:v>107</x:v>
       </x:c>
       <x:c r="O12" s="11" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P12" s="11" t="n">
+        <x:f>ROUND(O12*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q12" s="11" t="n">
+        <x:f>ROUND(O12*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R12" s="11" t="n">
+        <x:f>ROUND(O12*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S12" s="11" t="n">
@@ -52958,36 +53039,45 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="H13" s="15" t="n">
+        <x:f>ROUND(G13*1.5,0)</x:f>
         <x:v>900</x:v>
       </x:c>
       <x:c r="I13" s="15" t="n">
+        <x:f>ROUND(G13*3,0)</x:f>
         <x:v>1800</x:v>
       </x:c>
       <x:c r="J13" s="15" t="n">
+        <x:f>ROUND(G13*(3*1.15),0)</x:f>
         <x:v>2070</x:v>
       </x:c>
       <x:c r="K13" s="15" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="L13" s="15" t="n">
+        <x:f>ROUND(K13*1.5,0)</x:f>
         <x:v>39</x:v>
       </x:c>
       <x:c r="M13" s="15" t="n">
+        <x:f>ROUND(K13*3,0)</x:f>
         <x:v>78</x:v>
       </x:c>
       <x:c r="N13" s="15" t="n">
+        <x:f>ROUND(K13*(3*1.15),0)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="O13" s="15" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P13" s="15" t="n">
+        <x:f>ROUND(O13*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q13" s="15" t="n">
+        <x:f>ROUND(O13*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R13" s="15" t="n">
+        <x:f>ROUND(O13*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S13" s="15" t="n">
@@ -53045,36 +53135,45 @@
         <x:v>1080</x:v>
       </x:c>
       <x:c r="H14" s="11" t="n">
+        <x:f>ROUND(G14*1.5,0)</x:f>
         <x:v>1620</x:v>
       </x:c>
       <x:c r="I14" s="11" t="n">
+        <x:f>ROUND(G14*3,0)</x:f>
         <x:v>3240</x:v>
       </x:c>
       <x:c r="J14" s="11" t="n">
+        <x:f>ROUND(G14*(3*1.15),0)</x:f>
         <x:v>3726</x:v>
       </x:c>
       <x:c r="K14" s="11" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="L14" s="11" t="n">
+        <x:f>ROUND(K14*1.5,0)</x:f>
         <x:v>72</x:v>
       </x:c>
       <x:c r="M14" s="11" t="n">
+        <x:f>ROUND(K14*3,0)</x:f>
         <x:v>144</x:v>
       </x:c>
       <x:c r="N14" s="11" t="n">
+        <x:f>ROUND(K14*(3*1.15),0)</x:f>
         <x:v>166</x:v>
       </x:c>
       <x:c r="O14" s="11" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="P14" s="11" t="n">
+        <x:f>ROUND(O14*1.5,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="Q14" s="11" t="n">
+        <x:f>ROUND(O14*3,0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="R14" s="11" t="n">
+        <x:f>ROUND(O14*(3*1.15),0)</x:f>
         <x:v>28</x:v>
       </x:c>
       <x:c r="S14" s="11" t="n">
@@ -53132,36 +53231,45 @@
         <x:v>1040</x:v>
       </x:c>
       <x:c r="H15" s="15" t="n">
+        <x:f>ROUND(G15*1.5,0)</x:f>
         <x:v>1560</x:v>
       </x:c>
       <x:c r="I15" s="15" t="n">
+        <x:f>ROUND(G15*3,0)</x:f>
         <x:v>3120</x:v>
       </x:c>
       <x:c r="J15" s="15" t="n">
+        <x:f>ROUND(G15*(3*1.15),0)</x:f>
         <x:v>3588</x:v>
       </x:c>
       <x:c r="K15" s="15" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="L15" s="15" t="n">
+        <x:f>ROUND(K15*1.5,0)</x:f>
         <x:v>119</x:v>
       </x:c>
       <x:c r="M15" s="15" t="n">
+        <x:f>ROUND(K15*3,0)</x:f>
         <x:v>237</x:v>
       </x:c>
       <x:c r="N15" s="15" t="n">
+        <x:f>ROUND(K15*(3*1.15),0)</x:f>
         <x:v>273</x:v>
       </x:c>
       <x:c r="O15" s="15" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="P15" s="15" t="n">
+        <x:f>ROUND(O15*1.5,0)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="Q15" s="15" t="n">
+        <x:f>ROUND(O15*3,0)</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="R15" s="15" t="n">
+        <x:f>ROUND(O15*(3*1.15),0)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="S15" s="15" t="n">
@@ -53219,36 +53327,45 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="H16" s="11" t="n">
+        <x:f>ROUND(G16*1.5,0)</x:f>
         <x:v>1080</x:v>
       </x:c>
       <x:c r="I16" s="11" t="n">
+        <x:f>ROUND(G16*3,0)</x:f>
         <x:v>2160</x:v>
       </x:c>
       <x:c r="J16" s="11" t="n">
+        <x:f>ROUND(G16*(3*1.15),0)</x:f>
         <x:v>2484</x:v>
       </x:c>
       <x:c r="K16" s="11" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="L16" s="11" t="n">
+        <x:f>ROUND(K16*1.5,0)</x:f>
         <x:v>116</x:v>
       </x:c>
       <x:c r="M16" s="11" t="n">
+        <x:f>ROUND(K16*3,0)</x:f>
         <x:v>231</x:v>
       </x:c>
       <x:c r="N16" s="11" t="n">
+        <x:f>ROUND(K16*(3*1.15),0)</x:f>
         <x:v>266</x:v>
       </x:c>
       <x:c r="O16" s="11" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P16" s="11" t="n">
+        <x:f>ROUND(O16*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q16" s="11" t="n">
+        <x:f>ROUND(O16*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R16" s="11" t="n">
+        <x:f>ROUND(O16*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S16" s="11" t="n">
@@ -53306,36 +53423,45 @@
         <x:v>1520</x:v>
       </x:c>
       <x:c r="H17" s="15" t="n">
+        <x:f>ROUND(G17*1.5,0)</x:f>
         <x:v>2280</x:v>
       </x:c>
       <x:c r="I17" s="15" t="n">
+        <x:f>ROUND(G17*3,0)</x:f>
         <x:v>4560</x:v>
       </x:c>
       <x:c r="J17" s="15" t="n">
+        <x:f>ROUND(G17*(3*1.15),0)</x:f>
         <x:v>5244</x:v>
       </x:c>
       <x:c r="K17" s="15" t="n">
         <x:v>46</x:v>
       </x:c>
       <x:c r="L17" s="15" t="n">
+        <x:f>ROUND(K17*1.5,0)</x:f>
         <x:v>69</x:v>
       </x:c>
       <x:c r="M17" s="15" t="n">
+        <x:f>ROUND(K17*3,0)</x:f>
         <x:v>138</x:v>
       </x:c>
       <x:c r="N17" s="15" t="n">
+        <x:f>ROUND(K17*(3*1.15),0)</x:f>
         <x:v>159</x:v>
       </x:c>
       <x:c r="O17" s="15" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="P17" s="15" t="n">
+        <x:f>ROUND(O17*1.5,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="Q17" s="15" t="n">
+        <x:f>ROUND(O17*3,0)</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="R17" s="15" t="n">
+        <x:f>ROUND(O17*(3*1.15),0)</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="S17" s="15" t="n">
@@ -53393,36 +53519,45 @@
         <x:v>1700</x:v>
       </x:c>
       <x:c r="H18" s="11" t="n">
+        <x:f>ROUND(G18*1.5,0)</x:f>
         <x:v>2550</x:v>
       </x:c>
       <x:c r="I18" s="11" t="n">
+        <x:f>ROUND(G18*3,0)</x:f>
         <x:v>5100</x:v>
       </x:c>
       <x:c r="J18" s="11" t="n">
+        <x:f>ROUND(G18*(3*1.15),0)</x:f>
         <x:v>5865</x:v>
       </x:c>
       <x:c r="K18" s="11" t="n">
         <x:v>73</x:v>
       </x:c>
       <x:c r="L18" s="11" t="n">
+        <x:f>ROUND(K18*1.5,0)</x:f>
         <x:v>110</x:v>
       </x:c>
       <x:c r="M18" s="11" t="n">
+        <x:f>ROUND(K18*3,0)</x:f>
         <x:v>219</x:v>
       </x:c>
       <x:c r="N18" s="11" t="n">
+        <x:f>ROUND(K18*(3*1.15),0)</x:f>
         <x:v>252</x:v>
       </x:c>
       <x:c r="O18" s="11" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="P18" s="11" t="n">
+        <x:f>ROUND(O18*1.5,0)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="Q18" s="11" t="n">
+        <x:f>ROUND(O18*3,0)</x:f>
         <x:v>45</x:v>
       </x:c>
       <x:c r="R18" s="11" t="n">
+        <x:f>ROUND(O18*(3*1.15),0)</x:f>
         <x:v>52</x:v>
       </x:c>
       <x:c r="S18" s="11" t="n">
@@ -53482,36 +53617,45 @@
         <x:v>1800</x:v>
       </x:c>
       <x:c r="H19" s="15" t="n">
+        <x:f>ROUND(G19*1.5,0)</x:f>
         <x:v>2700</x:v>
       </x:c>
       <x:c r="I19" s="15" t="n">
+        <x:f>ROUND(G19*3,0)</x:f>
         <x:v>5400</x:v>
       </x:c>
       <x:c r="J19" s="15" t="n">
+        <x:f>ROUND(G19*(3*1.15),0)</x:f>
         <x:v>6210</x:v>
       </x:c>
       <x:c r="K19" s="15" t="n">
         <x:v>105</x:v>
       </x:c>
       <x:c r="L19" s="15" t="n">
+        <x:f>ROUND(K19*1.5,0)</x:f>
         <x:v>158</x:v>
       </x:c>
       <x:c r="M19" s="15" t="n">
+        <x:f>ROUND(K19*3,0)</x:f>
         <x:v>315</x:v>
       </x:c>
       <x:c r="N19" s="15" t="n">
+        <x:f>ROUND(K19*(3*1.15),0)</x:f>
         <x:v>362</x:v>
       </x:c>
       <x:c r="O19" s="15" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="P19" s="15" t="n">
+        <x:f>ROUND(O19*1.5,0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="Q19" s="15" t="n">
+        <x:f>ROUND(O19*3,0)</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="R19" s="15" t="n">
+        <x:f>ROUND(O19*(3*1.15),0)</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="S19" s="15" t="n">
@@ -53571,36 +53715,45 @@
         <x:v>560</x:v>
       </x:c>
       <x:c r="H20" s="11" t="n">
+        <x:f>ROUND(G20*1.5,0)</x:f>
         <x:v>840</x:v>
       </x:c>
       <x:c r="I20" s="11" t="n">
+        <x:f>ROUND(G20*3,0)</x:f>
         <x:v>1680</x:v>
       </x:c>
       <x:c r="J20" s="11" t="n">
+        <x:f>ROUND(G20*(3*1.15),0)</x:f>
         <x:v>1932</x:v>
       </x:c>
       <x:c r="K20" s="11" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="L20" s="11" t="n">
+        <x:f>ROUND(K20*1.5,0)</x:f>
         <x:v>44</x:v>
       </x:c>
       <x:c r="M20" s="11" t="n">
+        <x:f>ROUND(K20*3,0)</x:f>
         <x:v>87</x:v>
       </x:c>
       <x:c r="N20" s="11" t="n">
+        <x:f>ROUND(K20*(3*1.15),0)</x:f>
         <x:v>100</x:v>
       </x:c>
       <x:c r="O20" s="11" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P20" s="11" t="n">
+        <x:f>ROUND(O20*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q20" s="11" t="n">
+        <x:f>ROUND(O20*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R20" s="11" t="n">
+        <x:f>ROUND(O20*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S20" s="11" t="n">
@@ -53658,36 +53811,45 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="H21" s="15" t="n">
+        <x:f>ROUND(G21*1.5,0)</x:f>
         <x:v>900</x:v>
       </x:c>
       <x:c r="I21" s="15" t="n">
+        <x:f>ROUND(G21*3,0)</x:f>
         <x:v>1800</x:v>
       </x:c>
       <x:c r="J21" s="15" t="n">
+        <x:f>ROUND(G21*(3*1.15),0)</x:f>
         <x:v>2070</x:v>
       </x:c>
       <x:c r="K21" s="15" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="L21" s="15" t="n">
+        <x:f>ROUND(K21*1.5,0)</x:f>
         <x:v>53</x:v>
       </x:c>
       <x:c r="M21" s="15" t="n">
+        <x:f>ROUND(K21*3,0)</x:f>
         <x:v>105</x:v>
       </x:c>
       <x:c r="N21" s="15" t="n">
+        <x:f>ROUND(K21*(3*1.15),0)</x:f>
         <x:v>121</x:v>
       </x:c>
       <x:c r="O21" s="15" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="P21" s="15" t="n">
+        <x:f>ROUND(O21*1.5,0)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="Q21" s="15" t="n">
+        <x:f>ROUND(O21*3,0)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="R21" s="15" t="n">
+        <x:f>ROUND(O21*(3*1.15),0)</x:f>
         <x:v>17</x:v>
       </x:c>
       <x:c r="S21" s="15" t="n">
@@ -53745,36 +53907,45 @@
         <x:v>760</x:v>
       </x:c>
       <x:c r="H22" s="11" t="n">
+        <x:f>ROUND(G22*1.5,0)</x:f>
         <x:v>1140</x:v>
       </x:c>
       <x:c r="I22" s="11" t="n">
+        <x:f>ROUND(G22*3,0)</x:f>
         <x:v>2280</x:v>
       </x:c>
       <x:c r="J22" s="11" t="n">
+        <x:f>ROUND(G22*(3*1.15),0)</x:f>
         <x:v>2622</x:v>
       </x:c>
       <x:c r="K22" s="11" t="n">
         <x:v>70</x:v>
       </x:c>
       <x:c r="L22" s="11" t="n">
+        <x:f>ROUND(K22*1.5,0)</x:f>
         <x:v>105</x:v>
       </x:c>
       <x:c r="M22" s="11" t="n">
+        <x:f>ROUND(K22*3,0)</x:f>
         <x:v>210</x:v>
       </x:c>
       <x:c r="N22" s="11" t="n">
+        <x:f>ROUND(K22*(3*1.15),0)</x:f>
         <x:v>241</x:v>
       </x:c>
       <x:c r="O22" s="11" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="P22" s="11" t="n">
+        <x:f>ROUND(O22*1.5,0)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q22" s="11" t="n">
+        <x:f>ROUND(O22*3,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="R22" s="11" t="n">
+        <x:f>ROUND(O22*(3*1.15),0)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="S22" s="11" t="n">
@@ -53832,36 +54003,45 @@
         <x:v>1200</x:v>
       </x:c>
       <x:c r="H23" s="15" t="n">
+        <x:f>ROUND(G23*1.5,0)</x:f>
         <x:v>1800</x:v>
       </x:c>
       <x:c r="I23" s="15" t="n">
+        <x:f>ROUND(G23*3,0)</x:f>
         <x:v>3600</x:v>
       </x:c>
       <x:c r="J23" s="15" t="n">
+        <x:f>ROUND(G23*(3*1.15),0)</x:f>
         <x:v>4140</x:v>
       </x:c>
       <x:c r="K23" s="15" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="L23" s="15" t="n">
+        <x:f>ROUND(K23*1.5,0)</x:f>
         <x:v>72</x:v>
       </x:c>
       <x:c r="M23" s="15" t="n">
+        <x:f>ROUND(K23*3,0)</x:f>
         <x:v>144</x:v>
       </x:c>
       <x:c r="N23" s="15" t="n">
+        <x:f>ROUND(K23*(3*1.15),0)</x:f>
         <x:v>166</x:v>
       </x:c>
       <x:c r="O23" s="15" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="P23" s="15" t="n">
+        <x:f>ROUND(O23*1.5,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="Q23" s="15" t="n">
+        <x:f>ROUND(O23*3,0)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="R23" s="15" t="n">
+        <x:f>ROUND(O23*(3*1.15),0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="S23" s="15" t="n">
@@ -53919,36 +54099,45 @@
         <x:v>1640</x:v>
       </x:c>
       <x:c r="H24" s="11" t="n">
+        <x:f>ROUND(G24*1.5,0)</x:f>
         <x:v>2460</x:v>
       </x:c>
       <x:c r="I24" s="11" t="n">
+        <x:f>ROUND(G24*3,0)</x:f>
         <x:v>4920</x:v>
       </x:c>
       <x:c r="J24" s="11" t="n">
+        <x:f>ROUND(G24*(3*1.15),0)</x:f>
         <x:v>5658</x:v>
       </x:c>
       <x:c r="K24" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="L24" s="11" t="n">
+        <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="M24" s="11" t="n">
+        <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="N24" s="11" t="n">
+        <x:f>1</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="O24" s="11" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="P24" s="11" t="n">
+        <x:f>ROUND(O24*1.5,0)</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="Q24" s="11" t="n">
+        <x:f>ROUND(O24*3,0)</x:f>
         <x:v>54</x:v>
       </x:c>
       <x:c r="R24" s="11" t="n">
+        <x:f>ROUND(O24*(3*1.15),0)</x:f>
         <x:v>62</x:v>
       </x:c>
       <x:c r="S24" s="11" t="n">
@@ -54006,36 +54195,45 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="H25" s="15" t="n">
+        <x:f>ROUND(G25*1.5,0)</x:f>
         <x:v>1080</x:v>
       </x:c>
       <x:c r="I25" s="15" t="n">
+        <x:f>ROUND(G25*3,0)</x:f>
         <x:v>2160</x:v>
       </x:c>
       <x:c r="J25" s="15" t="n">
+        <x:f>ROUND(G25*(3*1.15),0)</x:f>
         <x:v>2484</x:v>
       </x:c>
       <x:c r="K25" s="15" t="n">
         <x:v>72</x:v>
       </x:c>
       <x:c r="L25" s="15" t="n">
+        <x:f>ROUND(K25*1.5,0)</x:f>
         <x:v>108</x:v>
       </x:c>
       <x:c r="M25" s="15" t="n">
+        <x:f>ROUND(K25*3,0)</x:f>
         <x:v>216</x:v>
       </x:c>
       <x:c r="N25" s="15" t="n">
+        <x:f>ROUND(K25*(3*1.15),0)</x:f>
         <x:v>248</x:v>
       </x:c>
       <x:c r="O25" s="15" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="P25" s="15" t="n">
+        <x:f>ROUND(O25*1.5,0)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q25" s="15" t="n">
+        <x:f>ROUND(O25*3,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="R25" s="15" t="n">
+        <x:f>ROUND(O25*(3*1.15),0)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="S25" s="15" t="n">
@@ -54093,36 +54291,45 @@
         <x:v>1120</x:v>
       </x:c>
       <x:c r="H26" s="11" t="n">
+        <x:f>ROUND(G26*1.5,0)</x:f>
         <x:v>1680</x:v>
       </x:c>
       <x:c r="I26" s="11" t="n">
+        <x:f>ROUND(G26*3,0)</x:f>
         <x:v>3360</x:v>
       </x:c>
       <x:c r="J26" s="11" t="n">
+        <x:f>ROUND(G26*(3*1.15),0)</x:f>
         <x:v>3864</x:v>
       </x:c>
       <x:c r="K26" s="11" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="L26" s="11" t="n">
+        <x:f>ROUND(K26*1.5,0)</x:f>
         <x:v>96</x:v>
       </x:c>
       <x:c r="M26" s="11" t="n">
+        <x:f>ROUND(K26*3,0)</x:f>
         <x:v>192</x:v>
       </x:c>
       <x:c r="N26" s="11" t="n">
+        <x:f>ROUND(K26*(3*1.15),0)</x:f>
         <x:v>221</x:v>
       </x:c>
       <x:c r="O26" s="11" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="P26" s="11" t="n">
+        <x:f>ROUND(O26*1.5,0)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="Q26" s="11" t="n">
+        <x:f>ROUND(O26*3,0)</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="R26" s="11" t="n">
+        <x:f>ROUND(O26*(3*1.15),0)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="S26" s="11" t="n">
@@ -54180,36 +54387,45 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="H27" s="15" t="n">
+        <x:f>ROUND(G27*1.5,0)</x:f>
         <x:v>1080</x:v>
       </x:c>
       <x:c r="I27" s="15" t="n">
+        <x:f>ROUND(G27*3,0)</x:f>
         <x:v>2160</x:v>
       </x:c>
       <x:c r="J27" s="15" t="n">
+        <x:f>ROUND(G27*(3*1.15),0)</x:f>
         <x:v>2484</x:v>
       </x:c>
       <x:c r="K27" s="15" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="L27" s="15" t="n">
+        <x:f>ROUND(K27*1.5,0)</x:f>
         <x:v>83</x:v>
       </x:c>
       <x:c r="M27" s="15" t="n">
+        <x:f>ROUND(K27*3,0)</x:f>
         <x:v>165</x:v>
       </x:c>
       <x:c r="N27" s="15" t="n">
+        <x:f>ROUND(K27*(3*1.15),0)</x:f>
         <x:v>190</x:v>
       </x:c>
       <x:c r="O27" s="15" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="P27" s="15" t="n">
+        <x:f>ROUND(O27*1.5,0)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="Q27" s="15" t="n">
+        <x:f>ROUND(O27*3,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="R27" s="15" t="n">
+        <x:f>ROUND(O27*(3*1.15),0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="S27" s="15" t="n">
@@ -54269,36 +54485,45 @@
         <x:v>660</x:v>
       </x:c>
       <x:c r="H28" s="11" t="n">
+        <x:f>ROUND(G28*1.5,0)</x:f>
         <x:v>990</x:v>
       </x:c>
       <x:c r="I28" s="11" t="n">
+        <x:f>ROUND(G28*3,0)</x:f>
         <x:v>1980</x:v>
       </x:c>
       <x:c r="J28" s="11" t="n">
+        <x:f>ROUND(G28*(3*1.15),0)</x:f>
         <x:v>2277</x:v>
       </x:c>
       <x:c r="K28" s="11" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="L28" s="11" t="n">
+        <x:f>ROUND(K28*1.5,0)</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="M28" s="11" t="n">
+        <x:f>ROUND(K28*3,0)</x:f>
         <x:v>99</x:v>
       </x:c>
       <x:c r="N28" s="11" t="n">
+        <x:f>ROUND(K28*(3*1.15),0)</x:f>
         <x:v>114</x:v>
       </x:c>
       <x:c r="O28" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="P28" s="11" t="n">
+        <x:f>ROUND(O28*1.5,0)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="Q28" s="11" t="n">
+        <x:f>ROUND(O28*3,0)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="R28" s="11" t="n">
+        <x:f>ROUND(O28*(3*1.15),0)</x:f>
         <x:v>17</x:v>
       </x:c>
       <x:c r="S28" s="11" t="n">
@@ -54356,36 +54581,45 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="H29" s="15" t="n">
+        <x:f>ROUND(G29*1.5,0)</x:f>
         <x:v>900</x:v>
       </x:c>
       <x:c r="I29" s="15" t="n">
+        <x:f>ROUND(G29*3,0)</x:f>
         <x:v>1800</x:v>
       </x:c>
       <x:c r="J29" s="15" t="n">
+        <x:f>ROUND(G29*(3*1.5),0)</x:f>
         <x:v>2700</x:v>
       </x:c>
       <x:c r="K29" s="15" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="L29" s="15" t="n">
+        <x:f>ROUND(K29*1.5,0)</x:f>
         <x:v>36</x:v>
       </x:c>
       <x:c r="M29" s="15" t="n">
+        <x:f>ROUND(K29*3,0)</x:f>
         <x:v>72</x:v>
       </x:c>
       <x:c r="N29" s="15" t="n">
+        <x:f>ROUND(K29*(3*1.5),0)</x:f>
         <x:v>108</x:v>
       </x:c>
       <x:c r="O29" s="15" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="P29" s="15" t="n">
+        <x:f>ROUND(O29*1.5,0)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q29" s="15" t="n">
+        <x:f>ROUND(O29*3,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="R29" s="15" t="n">
+        <x:f>ROUND(O29*(3*1.5),0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="S29" s="15" t="n">
@@ -54443,36 +54677,45 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="H30" s="11" t="n">
+        <x:f>ROUND(G30*1.5,0)</x:f>
         <x:v>900</x:v>
       </x:c>
       <x:c r="I30" s="11" t="n">
+        <x:f>ROUND(G30*3,0)</x:f>
         <x:v>1800</x:v>
       </x:c>
       <x:c r="J30" s="11" t="n">
+        <x:f>ROUND(G30*(3*1.15),0)</x:f>
         <x:v>2070</x:v>
       </x:c>
       <x:c r="K30" s="11" t="n">
         <x:v>145</x:v>
       </x:c>
       <x:c r="L30" s="11" t="n">
+        <x:f>ROUND(K30*1.5,0)</x:f>
         <x:v>218</x:v>
       </x:c>
       <x:c r="M30" s="11" t="n">
+        <x:f>ROUND(K30*3,0)</x:f>
         <x:v>435</x:v>
       </x:c>
       <x:c r="N30" s="11" t="n">
+        <x:f>ROUND(K30*(3*1.15),0)</x:f>
         <x:v>500</x:v>
       </x:c>
       <x:c r="O30" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P30" s="11" t="n">
+        <x:f>ROUND(O30*1.5,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q30" s="11" t="n">
+        <x:f>ROUND(O30*3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R30" s="11" t="n">
+        <x:f>ROUND(O30*(3*1.15),0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S30" s="11" t="n">
@@ -54530,36 +54773,45 @@
         <x:v>760</x:v>
       </x:c>
       <x:c r="H31" s="15" t="n">
+        <x:f>ROUND(G31*1.5,0)</x:f>
         <x:v>1140</x:v>
       </x:c>
       <x:c r="I31" s="15" t="n">
+        <x:f>ROUND(G31*3,0)</x:f>
         <x:v>2280</x:v>
       </x:c>
       <x:c r="J31" s="15" t="n">
+        <x:f>ROUND(G31*(3*1.15),0)</x:f>
         <x:v>2622</x:v>
       </x:c>
       <x:c r="K31" s="15" t="n">
         <x:v>66</x:v>
       </x:c>
       <x:c r="L31" s="15" t="n">
+        <x:f>ROUND(K31*1.5,0)</x:f>
         <x:v>99</x:v>
       </x:c>
       <x:c r="M31" s="15" t="n">
+        <x:f>ROUND(K31*3,0)</x:f>
         <x:v>198</x:v>
       </x:c>
       <x:c r="N31" s="15" t="n">
+        <x:f>ROUND(K31*(3*1.15),0)</x:f>
         <x:v>228</x:v>
       </x:c>
       <x:c r="O31" s="15" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P31" s="15" t="n">
+        <x:f>ROUND(O31*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q31" s="15" t="n">
+        <x:f>ROUND(O31*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R31" s="15" t="n">
+        <x:f>ROUND(O31*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S31" s="15" t="n">
@@ -54617,36 +54869,45 @@
         <x:v>840</x:v>
       </x:c>
       <x:c r="H32" s="11" t="n">
+        <x:f>ROUND(G32*1.5,0)</x:f>
         <x:v>1260</x:v>
       </x:c>
       <x:c r="I32" s="11" t="n">
+        <x:f>ROUND(G32*3,0)</x:f>
         <x:v>2520</x:v>
       </x:c>
       <x:c r="J32" s="11" t="n">
+        <x:f>ROUND(G32*(3*1.15),0)</x:f>
         <x:v>2898</x:v>
       </x:c>
       <x:c r="K32" s="11" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="L32" s="11" t="n">
+        <x:f>ROUND(K32*1.5,0)</x:f>
         <x:v>86</x:v>
       </x:c>
       <x:c r="M32" s="11" t="n">
+        <x:f>ROUND(K32*3,0)</x:f>
         <x:v>171</x:v>
       </x:c>
       <x:c r="N32" s="11" t="n">
+        <x:f>ROUND(K32*(3*1.15),0)</x:f>
         <x:v>197</x:v>
       </x:c>
       <x:c r="O32" s="11" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="P32" s="11" t="n">
+        <x:f>ROUND(O32*1.5,0)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="Q32" s="11" t="n">
+        <x:f>ROUND(O32*3,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="R32" s="11" t="n">
+        <x:f>ROUND(O32*(3*1.15),0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="S32" s="11" t="n">
@@ -54704,36 +54965,45 @@
         <x:v>800</x:v>
       </x:c>
       <x:c r="H33" s="15" t="n">
+        <x:f>ROUND(G33*1.5,0)</x:f>
         <x:v>1200</x:v>
       </x:c>
       <x:c r="I33" s="15" t="n">
+        <x:f>ROUND(G33*3,0)</x:f>
         <x:v>2400</x:v>
       </x:c>
       <x:c r="J33" s="15" t="n">
+        <x:f>ROUND(G33*(3*1.15),0)</x:f>
         <x:v>2760</x:v>
       </x:c>
       <x:c r="K33" s="15" t="n">
         <x:v>62</x:v>
       </x:c>
       <x:c r="L33" s="15" t="n">
+        <x:f>ROUND(K33*1.5,0)</x:f>
         <x:v>93</x:v>
       </x:c>
       <x:c r="M33" s="15" t="n">
+        <x:f>ROUND(K33*3,0)</x:f>
         <x:v>186</x:v>
       </x:c>
       <x:c r="N33" s="15" t="n">
+        <x:f>ROUND(K33*(3*1.15),0)</x:f>
         <x:v>214</x:v>
       </x:c>
       <x:c r="O33" s="15" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="P33" s="15" t="n">
+        <x:f>ROUND(O33*1.5,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="Q33" s="15" t="n">
+        <x:f>ROUND(O33*3,0)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="R33" s="15" t="n">
+        <x:f>ROUND(O33*(3*1.15),0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="S33" s="15" t="n">
@@ -54791,36 +55061,45 @@
         <x:v>1500</x:v>
       </x:c>
       <x:c r="H34" s="11" t="n">
+        <x:f>ROUND(G34*1.5,0)</x:f>
         <x:v>2250</x:v>
       </x:c>
       <x:c r="I34" s="11" t="n">
+        <x:f>ROUND(G34*3,0)</x:f>
         <x:v>4500</x:v>
       </x:c>
       <x:c r="J34" s="11" t="n">
+        <x:f>ROUND(G34*(3*1.15),0)</x:f>
         <x:v>5175</x:v>
       </x:c>
       <x:c r="K34" s="11" t="n">
         <x:v>50</x:v>
       </x:c>
       <x:c r="L34" s="11" t="n">
+        <x:f>ROUND(K34*1.5,0)</x:f>
         <x:v>75</x:v>
       </x:c>
       <x:c r="M34" s="11" t="n">
+        <x:f>ROUND(K34*3,0)</x:f>
         <x:v>150</x:v>
       </x:c>
       <x:c r="N34" s="11" t="n">
+        <x:f>ROUND(K34*(3*1.15),0)</x:f>
         <x:v>173</x:v>
       </x:c>
       <x:c r="O34" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="P34" s="11" t="n">
+        <x:f>ROUND(O34*1.5,0)</x:f>
         <x:v>32</x:v>
       </x:c>
       <x:c r="Q34" s="11" t="n">
+        <x:f>ROUND(O34*3,0)</x:f>
         <x:v>63</x:v>
       </x:c>
       <x:c r="R34" s="11" t="n">
+        <x:f>ROUND(O34*(3*1.15),0)</x:f>
         <x:v>72</x:v>
       </x:c>
       <x:c r="S34" s="11" t="n">
@@ -54878,36 +55157,45 @@
         <x:v>1600</x:v>
       </x:c>
       <x:c r="H35" s="15" t="n">
+        <x:f>ROUND(G35*1.5,0)</x:f>
         <x:v>2400</x:v>
       </x:c>
       <x:c r="I35" s="15" t="n">
+        <x:f>ROUND(G35*3,0)</x:f>
         <x:v>4800</x:v>
       </x:c>
       <x:c r="J35" s="15" t="n">
+        <x:f>ROUND(G35*(3*1.15),0)</x:f>
         <x:v>5520</x:v>
       </x:c>
       <x:c r="K35" s="15" t="n">
         <x:v>110</x:v>
       </x:c>
       <x:c r="L35" s="15" t="n">
+        <x:f>ROUND(K35*1.5,0)</x:f>
         <x:v>165</x:v>
       </x:c>
       <x:c r="M35" s="15" t="n">
+        <x:f>ROUND(K35*3,0)</x:f>
         <x:v>330</x:v>
       </x:c>
       <x:c r="N35" s="15" t="n">
+        <x:f>ROUND(K35*(3*1.15),0)</x:f>
         <x:v>379</x:v>
       </x:c>
       <x:c r="O35" s="15" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="P35" s="15" t="n">
+        <x:f>ROUND(O35*1.5,0)</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="Q35" s="15" t="n">
+        <x:f>ROUND(O35*3,0)</x:f>
         <x:v>54</x:v>
       </x:c>
       <x:c r="R35" s="15" t="n">
+        <x:f>ROUND(O35*(3*1.15),0)</x:f>
         <x:v>62</x:v>
       </x:c>
       <x:c r="S35" s="15" t="n">
@@ -54967,36 +55255,45 @@
         <x:v>650</x:v>
       </x:c>
       <x:c r="H36" s="11" t="n">
+        <x:f>ROUND(G36*1.5,0)</x:f>
         <x:v>975</x:v>
       </x:c>
       <x:c r="I36" s="11" t="n">
+        <x:f>ROUND(G36*3,0)</x:f>
         <x:v>1950</x:v>
       </x:c>
       <x:c r="J36" s="11" t="n">
+        <x:f>ROUND(G36*(3*1.15),0)</x:f>
         <x:v>2243</x:v>
       </x:c>
       <x:c r="K36" s="11" t="n">
         <x:v>31</x:v>
       </x:c>
       <x:c r="L36" s="11" t="n">
+        <x:f>ROUND(K36*1.5,0)</x:f>
         <x:v>47</x:v>
       </x:c>
       <x:c r="M36" s="11" t="n">
+        <x:f>ROUND(K36*3,0)</x:f>
         <x:v>93</x:v>
       </x:c>
       <x:c r="N36" s="11" t="n">
+        <x:f>ROUND(K36*(3*1.15),0)</x:f>
         <x:v>107</x:v>
       </x:c>
       <x:c r="O36" s="11" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="P36" s="11" t="n">
+        <x:f>ROUND(O36*1.5,0)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="Q36" s="11" t="n">
+        <x:f>ROUND(O36*3,0)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="R36" s="11" t="n">
+        <x:f>ROUND(O36*(3*1.15),0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="S36" s="11" t="n">
@@ -55054,36 +55351,45 @@
         <x:v>540</x:v>
       </x:c>
       <x:c r="H37" s="15" t="n">
+        <x:f>ROUND(G37*1.5,0)</x:f>
         <x:v>810</x:v>
       </x:c>
       <x:c r="I37" s="15" t="n">
+        <x:f>ROUND(G37*3,0)</x:f>
         <x:v>1620</x:v>
       </x:c>
       <x:c r="J37" s="15" t="n">
+        <x:f>ROUND(G37*(3*1.15),0)</x:f>
         <x:v>1863</x:v>
       </x:c>
       <x:c r="K37" s="15" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="L37" s="15" t="n">
+        <x:f>ROUND(K37*1.5,0)</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="M37" s="15" t="n">
+        <x:f>ROUND(K37*3,0)</x:f>
         <x:v>84</x:v>
       </x:c>
       <x:c r="N37" s="15" t="n">
+        <x:f>ROUND(K37*(3*1.15),0)</x:f>
         <x:v>97</x:v>
       </x:c>
       <x:c r="O37" s="15" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="P37" s="15" t="n">
+        <x:f>ROUND(O37*1.5,0)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q37" s="15" t="n">
+        <x:f>ROUND(O37*3,0)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="R37" s="15" t="n">
+        <x:f>ROUND(O37*(3*1.15),0)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="S37" s="15" t="n">
@@ -55141,36 +55447,45 @@
         <x:v>980</x:v>
       </x:c>
       <x:c r="H38" s="11" t="n">
+        <x:f>ROUND(G38*1.5,0)</x:f>
         <x:v>1470</x:v>
       </x:c>
       <x:c r="I38" s="11" t="n">
+        <x:f>ROUND(G38*3,0)</x:f>
         <x:v>2940</x:v>
       </x:c>
       <x:c r="J38" s="11" t="n">
+        <x:f>ROUND(G38*(3*1.15),0)</x:f>
         <x:v>3381</x:v>
       </x:c>
       <x:c r="K38" s="11" t="n">
         <x:v>52</x:v>
       </x:c>
       <x:c r="L38" s="11" t="n">
+        <x:f>ROUND(K38*1.5,0)</x:f>
         <x:v>78</x:v>
       </x:c>
       <x:c r="M38" s="11" t="n">
+        <x:f>ROUND(K38*3,0)</x:f>
         <x:v>156</x:v>
       </x:c>
       <x:c r="N38" s="11" t="n">
+        <x:f>ROUND(K38*(3*1.15),0)</x:f>
         <x:v>179</x:v>
       </x:c>
       <x:c r="O38" s="11" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="P38" s="11" t="n">
+        <x:f>ROUND(O38*1.5,0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="Q38" s="11" t="n">
+        <x:f>ROUND(O38*3,0)</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="R38" s="11" t="n">
+        <x:f>ROUND(O38*(3*1.15),0)</x:f>
         <x:v>31</x:v>
       </x:c>
       <x:c r="S38" s="11" t="n">
@@ -55228,36 +55543,45 @@
         <x:v>760</x:v>
       </x:c>
       <x:c r="H39" s="15" t="n">
+        <x:f>ROUND(G39*1.5,0)</x:f>
         <x:v>1140</x:v>
       </x:c>
       <x:c r="I39" s="15" t="n">
+        <x:f>ROUND(G39*3,0)</x:f>
         <x:v>2280</x:v>
       </x:c>
       <x:c r="J39" s="15" t="n">
+        <x:f>ROUND(G39*(3*1.15),0)</x:f>
         <x:v>2622</x:v>
       </x:c>
       <x:c r="K39" s="15" t="n">
         <x:v>56</x:v>
       </x:c>
       <x:c r="L39" s="15" t="n">
+        <x:f>ROUND(K39*1.5,0)</x:f>
         <x:v>84</x:v>
       </x:c>
       <x:c r="M39" s="15" t="n">
+        <x:f>ROUND(K39*3,0)</x:f>
         <x:v>168</x:v>
       </x:c>
       <x:c r="N39" s="15" t="n">
+        <x:f>ROUND(K39*(3*1.15),0)</x:f>
         <x:v>193</x:v>
       </x:c>
       <x:c r="O39" s="15" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P39" s="15" t="n">
+        <x:f>ROUND(O39*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q39" s="15" t="n">
+        <x:f>ROUND(O39*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R39" s="15" t="n">
+        <x:f>ROUND(O39*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S39" s="15" t="n">
@@ -55315,36 +55639,45 @@
         <x:v>1180</x:v>
       </x:c>
       <x:c r="H40" s="11" t="n">
+        <x:f>ROUND(G40*1.5,0)</x:f>
         <x:v>1770</x:v>
       </x:c>
       <x:c r="I40" s="11" t="n">
+        <x:f>ROUND(G40*3,0)</x:f>
         <x:v>3540</x:v>
       </x:c>
       <x:c r="J40" s="11" t="n">
+        <x:f>ROUND(G40*(3*1.15),0)</x:f>
         <x:v>4071</x:v>
       </x:c>
       <x:c r="K40" s="11" t="n">
         <x:v>54</x:v>
       </x:c>
       <x:c r="L40" s="11" t="n">
+        <x:f>ROUND(K40*1.5,0)</x:f>
         <x:v>81</x:v>
       </x:c>
       <x:c r="M40" s="11" t="n">
+        <x:f>ROUND(K40*3,0)</x:f>
         <x:v>162</x:v>
       </x:c>
       <x:c r="N40" s="11" t="n">
+        <x:f>ROUND(K40*(3*1.15),0)</x:f>
         <x:v>186</x:v>
       </x:c>
       <x:c r="O40" s="11" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="P40" s="11" t="n">
+        <x:f>ROUND(O40*1.5,0)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="Q40" s="11" t="n">
+        <x:f>ROUND(O40*3,0)</x:f>
         <x:v>36</x:v>
       </x:c>
       <x:c r="R40" s="11" t="n">
+        <x:f>ROUND(O40*(3*1.15),0)</x:f>
         <x:v>41</x:v>
       </x:c>
       <x:c r="S40" s="11" t="n">
@@ -55402,36 +55735,45 @@
         <x:v>780</x:v>
       </x:c>
       <x:c r="H41" s="15" t="n">
+        <x:f>ROUND(G41*1.5,0)</x:f>
         <x:v>1170</x:v>
       </x:c>
       <x:c r="I41" s="15" t="n">
+        <x:f>ROUND(G41*3,0)</x:f>
         <x:v>2340</x:v>
       </x:c>
       <x:c r="J41" s="15" t="n">
+        <x:f>ROUND(G41*(3*1.15),0)</x:f>
         <x:v>2691</x:v>
       </x:c>
       <x:c r="K41" s="15" t="n">
         <x:v>68</x:v>
       </x:c>
       <x:c r="L41" s="15" t="n">
+        <x:f>ROUND(K41*1.5,0)</x:f>
         <x:v>102</x:v>
       </x:c>
       <x:c r="M41" s="15" t="n">
+        <x:f>ROUND(K41*3,0)</x:f>
         <x:v>204</x:v>
       </x:c>
       <x:c r="N41" s="15" t="n">
+        <x:f>ROUND(K41*(3*1.15),0)</x:f>
         <x:v>235</x:v>
       </x:c>
       <x:c r="O41" s="15" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="P41" s="15" t="n">
+        <x:f>ROUND(O41*1.5,0)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="Q41" s="15" t="n">
+        <x:f>ROUND(O41*3,0)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="R41" s="15" t="n">
+        <x:f>ROUND(O41*(3*1.15),0)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="S41" s="15" t="n">
@@ -55489,36 +55831,45 @@
         <x:v>1500</x:v>
       </x:c>
       <x:c r="H42" s="11" t="n">
+        <x:f>ROUND(G42*1.5,0)</x:f>
         <x:v>2250</x:v>
       </x:c>
       <x:c r="I42" s="11" t="n">
+        <x:f>ROUND(G42*3,0)</x:f>
         <x:v>4500</x:v>
       </x:c>
       <x:c r="J42" s="11" t="n">
+        <x:f>ROUND(G42*(3*1.15),0)</x:f>
         <x:v>5175</x:v>
       </x:c>
       <x:c r="K42" s="11" t="n">
         <x:v>104</x:v>
       </x:c>
       <x:c r="L42" s="11" t="n">
+        <x:f>ROUND(K42*1.5,0)</x:f>
         <x:v>156</x:v>
       </x:c>
       <x:c r="M42" s="11" t="n">
+        <x:f>ROUND(K42*3,0)</x:f>
         <x:v>312</x:v>
       </x:c>
       <x:c r="N42" s="11" t="n">
+        <x:f>ROUND(K42*(3*1.15),0)</x:f>
         <x:v>359</x:v>
       </x:c>
       <x:c r="O42" s="11" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="P42" s="11" t="n">
+        <x:f>ROUND(O42*1.5,0)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="Q42" s="11" t="n">
+        <x:f>ROUND(O42*3,0)</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="R42" s="11" t="n">
+        <x:f>ROUND(O42*(3*1.15),0)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="S42" s="11" t="n">
@@ -55576,36 +55927,45 @@
         <x:v>1720</x:v>
       </x:c>
       <x:c r="H43" s="15" t="n">
+        <x:f>ROUND(G43*1.5,0)</x:f>
         <x:v>2580</x:v>
       </x:c>
       <x:c r="I43" s="15" t="n">
+        <x:f>ROUND(G43*3,0)</x:f>
         <x:v>5160</x:v>
       </x:c>
       <x:c r="J43" s="15" t="n">
+        <x:f>ROUND(G43*(3*1.15),0)</x:f>
         <x:v>5934</x:v>
       </x:c>
       <x:c r="K43" s="15" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="L43" s="15" t="n">
+        <x:f>ROUND(K43*1.5,0)</x:f>
         <x:v>123</x:v>
       </x:c>
       <x:c r="M43" s="15" t="n">
+        <x:f>ROUND(K43*3,0)</x:f>
         <x:v>246</x:v>
       </x:c>
       <x:c r="N43" s="15" t="n">
+        <x:f>ROUND(K43*(3*1.15),0)</x:f>
         <x:v>283</x:v>
       </x:c>
       <x:c r="O43" s="15" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="P43" s="15" t="n">
+        <x:f>ROUND(O43*1.5,0)</x:f>
         <x:v>24</x:v>
       </x:c>
       <x:c r="Q43" s="15" t="n">
+        <x:f>ROUND(O43*3,0)</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="R43" s="15" t="n">
+        <x:f>ROUND(O43*(3*1.15),0)</x:f>
         <x:v>55</x:v>
       </x:c>
       <x:c r="S43" s="15" t="n">
@@ -55679,7 +56039,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>名称、货币和价格必须与 90_运行配置的 data/shop.json 一致。新商品先在本页与机器页登记，再导出运行目录。</x:v>
+        <x:v>商城商品由 data/shop.json 管理；此页与 JSON 保持一致，发布检查会核对名称、货币、价格及上架状态。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -58082,7 +58442,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>宠物效果与详细说明取指定新表；商品 ID、货币、价格和是否展示取 data/shop.json。服务端实际售卖目录及价格须上线前再核。</x:v>
+        <x:v>编辑 E 列效果百分比时，同步修改 F、N 列的说明百分比；工具会阻止文案与效果不一致。商品价格仍由 data/shop.json 管理。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -58844,7 +59204,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>16 只野怪的基础值与战斗探针结论；回合成长另见回合页。</x:v>
+        <x:v>编辑 E–G 列基础 HP / 攻击 / 防御；回合成长和技能机制由 data/pve/pve_monsters.json 管理。运行前执行同步工具。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -60000,7 +60360,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>9 种 Boss；R5/R10/R15/R20 数值沿用指定新表的本机运行结果。</x:v>
+        <x:v>编辑首场 HP / 攻击（D、E 列）和 R5 防御（O 列）；游戏 JSON 保存乘以 1.5 前的整数基础值。其余回合数值由公式按现有成长倍率推算。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -60136,41 +60496,55 @@
       <x:c r="E4" s="11" t="n">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="F4" s="11"/>
+      <x:c r="F4" s="11" t="n">
+        <x:f>O4</x:f>
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="G4" s="11" t="n">
+        <x:f>D4</x:f>
         <x:v>3300</x:v>
       </x:c>
       <x:c r="H4" s="11" t="n">
+        <x:f>ROUND(ROUND(D4/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>4785</x:v>
       </x:c>
       <x:c r="I4" s="11" t="n">
+        <x:f>ROUND(ROUND(D4/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>6938</x:v>
       </x:c>
       <x:c r="J4" s="11" t="n">
+        <x:f>ROUND(ROUND(D4/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>10060</x:v>
       </x:c>
       <x:c r="K4" s="11" t="n">
+        <x:f>E4</x:f>
         <x:v>113</x:v>
       </x:c>
       <x:c r="L4" s="11" t="n">
+        <x:f>ROUND(ROUND(E4/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>152</x:v>
       </x:c>
       <x:c r="M4" s="11" t="n">
+        <x:f>ROUND(ROUND(E4/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>205</x:v>
       </x:c>
       <x:c r="N4" s="11" t="n">
+        <x:f>ROUND(ROUND(E4/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>277</x:v>
       </x:c>
       <x:c r="O4" s="11" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="P4" s="11" t="n">
+        <x:f>ROUND(ROUND(O4/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="Q4" s="11" t="n">
+        <x:f>ROUND(ROUND(O4/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="R4" s="11" t="n">
+        <x:f>ROUND(ROUND(O4/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="S4" s="11" t="n">
@@ -60225,41 +60599,55 @@
       <x:c r="E5" s="15" t="n">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="F5" s="15"/>
+      <x:c r="F5" s="15" t="n">
+        <x:f>O5</x:f>
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="G5" s="15" t="n">
+        <x:f>D5</x:f>
         <x:v>3750</x:v>
       </x:c>
       <x:c r="H5" s="15" t="n">
+        <x:f>ROUND(ROUND(D5/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>5438</x:v>
       </x:c>
       <x:c r="I5" s="15" t="n">
+        <x:f>ROUND(ROUND(D5/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>7884</x:v>
       </x:c>
       <x:c r="J5" s="15" t="n">
+        <x:f>ROUND(ROUND(D5/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>11432</x:v>
       </x:c>
       <x:c r="K5" s="15" t="n">
+        <x:f>E5</x:f>
         <x:v>92</x:v>
       </x:c>
       <x:c r="L5" s="15" t="n">
+        <x:f>ROUND(ROUND(E5/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>124</x:v>
       </x:c>
       <x:c r="M5" s="15" t="n">
+        <x:f>ROUND(ROUND(E5/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>167</x:v>
       </x:c>
       <x:c r="N5" s="15" t="n">
+        <x:f>ROUND(ROUND(E5/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>225</x:v>
       </x:c>
       <x:c r="O5" s="15" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="P5" s="15" t="n">
+        <x:f>ROUND(ROUND(O5/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>29</x:v>
       </x:c>
       <x:c r="Q5" s="15" t="n">
+        <x:f>ROUND(ROUND(O5/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>38</x:v>
       </x:c>
       <x:c r="R5" s="15" t="n">
+        <x:f>ROUND(ROUND(O5/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>49</x:v>
       </x:c>
       <x:c r="S5" s="15" t="n">
@@ -60315,41 +60703,55 @@
       <x:c r="E6" s="11" t="n">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="F6" s="11"/>
+      <x:c r="F6" s="11" t="n">
+        <x:f>O6</x:f>
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="G6" s="11" t="n">
+        <x:f>D6</x:f>
         <x:v>2700</x:v>
       </x:c>
       <x:c r="H6" s="11" t="n">
+        <x:f>ROUND(ROUND(D6/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>3915</x:v>
       </x:c>
       <x:c r="I6" s="11" t="n">
+        <x:f>ROUND(ROUND(D6/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>5677</x:v>
       </x:c>
       <x:c r="J6" s="11" t="n">
+        <x:f>ROUND(ROUND(D6/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>8231</x:v>
       </x:c>
       <x:c r="K6" s="11" t="n">
+        <x:f>E6</x:f>
         <x:v>116</x:v>
       </x:c>
       <x:c r="L6" s="11" t="n">
+        <x:f>ROUND(ROUND(E6/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>156</x:v>
       </x:c>
       <x:c r="M6" s="11" t="n">
+        <x:f>ROUND(ROUND(E6/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>210</x:v>
       </x:c>
       <x:c r="N6" s="11" t="n">
+        <x:f>ROUND(ROUND(E6/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>284</x:v>
       </x:c>
       <x:c r="O6" s="11" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="P6" s="11" t="n">
+        <x:f>ROUND(ROUND(O6/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="Q6" s="11" t="n">
+        <x:f>ROUND(ROUND(O6/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="R6" s="11" t="n">
+        <x:f>ROUND(ROUND(O6/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>26</x:v>
       </x:c>
       <x:c r="S6" s="11" t="n">
@@ -60406,41 +60808,55 @@
       <x:c r="E7" s="15" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="F7" s="15"/>
+      <x:c r="F7" s="15" t="n">
+        <x:f>O7</x:f>
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="G7" s="15" t="n">
+        <x:f>D7</x:f>
         <x:v>3000</x:v>
       </x:c>
       <x:c r="H7" s="15" t="n">
+        <x:f>ROUND(ROUND(D7/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>4350</x:v>
       </x:c>
       <x:c r="I7" s="15" t="n">
+        <x:f>ROUND(ROUND(D7/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>6308</x:v>
       </x:c>
       <x:c r="J7" s="15" t="n">
+        <x:f>ROUND(ROUND(D7/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>9146</x:v>
       </x:c>
       <x:c r="K7" s="15" t="n">
+        <x:f>E7</x:f>
         <x:v>75</x:v>
       </x:c>
       <x:c r="L7" s="15" t="n">
+        <x:f>ROUND(ROUND(E7/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>101</x:v>
       </x:c>
       <x:c r="M7" s="15" t="n">
+        <x:f>ROUND(ROUND(E7/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>137</x:v>
       </x:c>
       <x:c r="N7" s="15" t="n">
+        <x:f>ROUND(ROUND(E7/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>185</x:v>
       </x:c>
       <x:c r="O7" s="15" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="P7" s="15" t="n">
+        <x:f>ROUND(ROUND(O7/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="Q7" s="15" t="n">
+        <x:f>ROUND(ROUND(O7/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="R7" s="15" t="n">
+        <x:f>ROUND(ROUND(O7/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="S7" s="15" t="n">
@@ -60496,41 +60912,55 @@
       <x:c r="E8" s="11" t="n">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="F8" s="11"/>
+      <x:c r="F8" s="11" t="n">
+        <x:f>O8</x:f>
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="G8" s="11" t="n">
+        <x:f>D8</x:f>
         <x:v>2850</x:v>
       </x:c>
       <x:c r="H8" s="11" t="n">
+        <x:f>ROUND(ROUND(D8/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>4133</x:v>
       </x:c>
       <x:c r="I8" s="11" t="n">
+        <x:f>ROUND(ROUND(D8/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>5992</x:v>
       </x:c>
       <x:c r="J8" s="11" t="n">
+        <x:f>ROUND(ROUND(D8/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>8689</x:v>
       </x:c>
       <x:c r="K8" s="11" t="n">
+        <x:f>E8</x:f>
         <x:v>83</x:v>
       </x:c>
       <x:c r="L8" s="11" t="n">
+        <x:f>ROUND(ROUND(E8/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>111</x:v>
       </x:c>
       <x:c r="M8" s="11" t="n">
+        <x:f>ROUND(ROUND(E8/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>150</x:v>
       </x:c>
       <x:c r="N8" s="11" t="n">
+        <x:f>ROUND(ROUND(E8/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>203</x:v>
       </x:c>
       <x:c r="O8" s="11" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="P8" s="11" t="n">
+        <x:f>ROUND(ROUND(O8/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="Q8" s="11" t="n">
+        <x:f>ROUND(ROUND(O8/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="R8" s="11" t="n">
+        <x:f>ROUND(ROUND(O8/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="S8" s="11" t="n">
@@ -60586,41 +61016,55 @@
       <x:c r="E9" s="15" t="n">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="F9" s="15"/>
+      <x:c r="F9" s="15" t="n">
+        <x:f>O9</x:f>
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="G9" s="15" t="n">
+        <x:f>D9</x:f>
         <x:v>3000</x:v>
       </x:c>
       <x:c r="H9" s="15" t="n">
+        <x:f>ROUND(ROUND(D9/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>4350</x:v>
       </x:c>
       <x:c r="I9" s="15" t="n">
+        <x:f>ROUND(ROUND(D9/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>6308</x:v>
       </x:c>
       <x:c r="J9" s="15" t="n">
+        <x:f>ROUND(ROUND(D9/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>9146</x:v>
       </x:c>
       <x:c r="K9" s="15" t="n">
+        <x:f>E9</x:f>
         <x:v>92</x:v>
       </x:c>
       <x:c r="L9" s="15" t="n">
+        <x:f>ROUND(ROUND(E9/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>124</x:v>
       </x:c>
       <x:c r="M9" s="15" t="n">
+        <x:f>ROUND(ROUND(E9/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>167</x:v>
       </x:c>
       <x:c r="N9" s="15" t="n">
+        <x:f>ROUND(ROUND(E9/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>225</x:v>
       </x:c>
       <x:c r="O9" s="15" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="P9" s="15" t="n">
+        <x:f>ROUND(ROUND(O9/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="Q9" s="15" t="n">
+        <x:f>ROUND(ROUND(O9/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>30</x:v>
       </x:c>
       <x:c r="R9" s="15" t="n">
+        <x:f>ROUND(ROUND(O9/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>40</x:v>
       </x:c>
       <x:c r="S9" s="15" t="n">
@@ -60677,41 +61121,55 @@
       <x:c r="E10" s="11" t="n">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="F10" s="11"/>
+      <x:c r="F10" s="11" t="n">
+        <x:f>O10</x:f>
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="G10" s="11" t="n">
+        <x:f>D10</x:f>
         <x:v>3150</x:v>
       </x:c>
       <x:c r="H10" s="11" t="n">
+        <x:f>ROUND(ROUND(D10/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>4568</x:v>
       </x:c>
       <x:c r="I10" s="11" t="n">
+        <x:f>ROUND(ROUND(D10/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>6623</x:v>
       </x:c>
       <x:c r="J10" s="11" t="n">
+        <x:f>ROUND(ROUND(D10/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>9603</x:v>
       </x:c>
       <x:c r="K10" s="11" t="n">
+        <x:f>E10</x:f>
         <x:v>119</x:v>
       </x:c>
       <x:c r="L10" s="11" t="n">
+        <x:f>ROUND(ROUND(E10/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>160</x:v>
       </x:c>
       <x:c r="M10" s="11" t="n">
+        <x:f>ROUND(ROUND(E10/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>216</x:v>
       </x:c>
       <x:c r="N10" s="11" t="n">
+        <x:f>ROUND(ROUND(E10/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>292</x:v>
       </x:c>
       <x:c r="O10" s="11" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="P10" s="11" t="n">
+        <x:f>ROUND(ROUND(O10/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="Q10" s="11" t="n">
+        <x:f>ROUND(ROUND(O10/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="R10" s="11" t="n">
+        <x:f>ROUND(ROUND(O10/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="S10" s="11" t="n">
@@ -60766,41 +61224,55 @@
       <x:c r="E11" s="15" t="n">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="F11" s="15"/>
+      <x:c r="F11" s="15" t="n">
+        <x:f>O11</x:f>
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="G11" s="15" t="n">
+        <x:f>D11</x:f>
         <x:v>2100</x:v>
       </x:c>
       <x:c r="H11" s="15" t="n">
+        <x:f>ROUND(ROUND(D11/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>3045</x:v>
       </x:c>
       <x:c r="I11" s="15" t="n">
+        <x:f>ROUND(ROUND(D11/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>4415</x:v>
       </x:c>
       <x:c r="J11" s="15" t="n">
+        <x:f>ROUND(ROUND(D11/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>6402</x:v>
       </x:c>
       <x:c r="K11" s="15" t="n">
+        <x:f>E11</x:f>
         <x:v>96</x:v>
       </x:c>
       <x:c r="L11" s="15" t="n">
+        <x:f>ROUND(ROUND(E11/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>130</x:v>
       </x:c>
       <x:c r="M11" s="15" t="n">
+        <x:f>ROUND(ROUND(E11/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>175</x:v>
       </x:c>
       <x:c r="N11" s="15" t="n">
+        <x:f>ROUND(ROUND(E11/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>236</x:v>
       </x:c>
       <x:c r="O11" s="15" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="P11" s="15" t="n">
+        <x:f>ROUND(ROUND(O11/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="Q11" s="15" t="n">
+        <x:f>ROUND(ROUND(O11/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="R11" s="15" t="n">
+        <x:f>ROUND(ROUND(O11/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>33</x:v>
       </x:c>
       <x:c r="S11" s="15" t="n">
@@ -60858,41 +61330,55 @@
       <x:c r="E12" s="11" t="n">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="F12" s="11"/>
+      <x:c r="F12" s="11" t="n">
+        <x:f>O12</x:f>
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="G12" s="11" t="n">
+        <x:f>D12</x:f>
         <x:v>4200</x:v>
       </x:c>
       <x:c r="H12" s="11" t="n">
+        <x:f>ROUND(ROUND(D12/1.5,0)*1.5*1.45,0)</x:f>
         <x:v>6090</x:v>
       </x:c>
       <x:c r="I12" s="11" t="n">
+        <x:f>ROUND(ROUND(D12/1.5,0)*1.5*2.1025,0)</x:f>
         <x:v>8831</x:v>
       </x:c>
       <x:c r="J12" s="11" t="n">
+        <x:f>ROUND(ROUND(D12/1.5,0)*1.5*3.048625,0)</x:f>
         <x:v>12804</x:v>
       </x:c>
       <x:c r="K12" s="11" t="n">
+        <x:f>E12</x:f>
         <x:v>99</x:v>
       </x:c>
       <x:c r="L12" s="11" t="n">
+        <x:f>ROUND(ROUND(E12/1.5,0)*1.5*1.35,0)</x:f>
         <x:v>134</x:v>
       </x:c>
       <x:c r="M12" s="11" t="n">
+        <x:f>ROUND(ROUND(E12/1.5,0)*1.5*1.8225,0)</x:f>
         <x:v>180</x:v>
       </x:c>
       <x:c r="N12" s="11" t="n">
+        <x:f>ROUND(ROUND(E12/1.5,0)*1.5*2.460375,0)</x:f>
         <x:v>244</x:v>
       </x:c>
       <x:c r="O12" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="P12" s="11" t="n">
+        <x:f>ROUND(ROUND(O12/1.5,0)*1.5*1.3,0)</x:f>
         <x:v>27</x:v>
       </x:c>
       <x:c r="Q12" s="11" t="n">
+        <x:f>ROUND(ROUND(O12/1.5,0)*1.5*1.69,0)</x:f>
         <x:v>35</x:v>
       </x:c>
       <x:c r="R12" s="11" t="n">
+        <x:f>ROUND(ROUND(O12/1.5,0)*1.5*2.197,0)</x:f>
         <x:v>46</x:v>
       </x:c>
       <x:c r="S12" s="11" t="n">
@@ -62089,7 +62575,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>最终回合按法阵生命召唤的 5 种友军。</x:v>
+        <x:v>编辑 E–G 列 HP / 攻击 / 防御；技能和召唤规则由 JSON / GDScript 管理。运行前执行同步工具。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>

</xml_diff>